<commit_message>
Momentum scan results 2026-08-22
</commit_message>
<xml_diff>
--- a/results/momentum_2026-08-22.xlsx
+++ b/results/momentum_2026-08-22.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -495,12 +495,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>BR</t>
+          <t>AVTR</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>BMNR</t>
+          <t>BNTX</t>
         </is>
       </c>
     </row>
@@ -517,12 +517,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>BTU</t>
+          <t>BETA</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>BRZE</t>
+          <t>CGAU</t>
         </is>
       </c>
     </row>
@@ -539,12 +539,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>CAKE</t>
+          <t>BSY</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>CAI</t>
+          <t>CSX</t>
         </is>
       </c>
     </row>
@@ -556,17 +556,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ARX</t>
+          <t>BLSH</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>CELH</t>
+          <t>CCC</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>CME</t>
+          <t>EXE</t>
         </is>
       </c>
     </row>
@@ -578,331 +578,347 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>AVTR</t>
+          <t>BMNR</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>CMCSA</t>
+          <t>CLBK</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>EXE</t>
+          <t>FBRX</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>BETA</t>
+          <t>ARX</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>BLSH</t>
+          <t>BRZE</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>DBX</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>FBRX</t>
+          <t>IBKR</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>BSY</t>
+          <t>SKHY</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>BNTX</t>
+          <t>CAI</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>DFTX</t>
+          <t>CTSH</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>IBKR</t>
+          <t>ILMN</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CCC</t>
+          <t>BR</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CGAU</t>
+          <t>CME</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>DXCM</t>
+          <t>DASH</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>ILMN</t>
+          <t>INFQ</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CLBK</t>
+          <t>BTU</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CSX</t>
+          <t>FUTU</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>FIVN</t>
+          <t>DKNG</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>INFQ</t>
+          <t>NDAQ</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>CAKE</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>FUTU</t>
+          <t>INTU</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>GEHC</t>
+          <t>DXCM</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>MKTX</t>
+          <t>PAA</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CTSH</t>
+          <t>CELH</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>INTU</t>
+          <t>MKTX</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>HALO</t>
+          <t>FIVN</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>PEP</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>DASH</t>
+          <t>CMCSA</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>NDAQ</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>MDLZ</t>
+          <t>GEHC</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>NTNX</t>
+          <t>RGEN</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>DKNG</t>
+          <t>DBX</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>PAGP</t>
+          <t>NTNX</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>OCUL</t>
+          <t>HALO</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>NVAX</t>
+          <t>ROIV</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>EXLS</t>
+          <t>DFTX</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>PEP</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr"/>
+          <t>NVAX</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>MDLZ</t>
+        </is>
+      </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>PAA</t>
+          <t>SBLK</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>FIGR</t>
+          <t>EXLS</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>PLTR</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr"/>
+          <t>PAGP</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>OCUL</t>
+        </is>
+      </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>RGEN</t>
+          <t>SOFI</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>FROG</t>
+          <t>FIGR</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>PSNL</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr"/>
+          <t>PLTR</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>SNY</t>
+        </is>
+      </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>ROIV</t>
+          <t>SSRM</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>GH</t>
+          <t>FROG</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>PURR</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr"/>
+          <t>PSNL</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>CPRT</t>
+        </is>
+      </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>SBLK</t>
+          <t>RELY</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>HTFL</t>
+          <t>GH</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>RVMD</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr"/>
+          <t>PURR</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>AVAH</t>
+        </is>
+      </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>SLS</t>
+          <t>ROKU</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>LYFT</t>
+          <t>HTFL</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>SBET</t>
+          <t>RVMD</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
-          <t>SSRM</t>
+          <t>HTHT</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>NTRA</t>
+          <t>LYFT</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>SOFI</t>
+          <t>SBET</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>TRMB</t>
-        </is>
-      </c>
+      <c r="D23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>NWSA</t>
+          <t>NTRA</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>SSNC</t>
+          <t>SLS</t>
         </is>
       </c>
       <c r="C24" t="inlineStr"/>
@@ -911,12 +927,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>OMER</t>
+          <t>NWSA</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>STRC</t>
+          <t>SSNC</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
@@ -925,12 +941,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>PAYX</t>
+          <t>OMER</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>TEM</t>
+          <t>STRC</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -939,12 +955,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>RELY</t>
+          <t>PAYX</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>TW</t>
+          <t>TEM</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -953,12 +969,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ROKU</t>
+          <t>PPC</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PPC</t>
+          <t>TW</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -967,12 +983,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>SHC</t>
+          <t>PTEN</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>PTEN</t>
+          <t>SHOP</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -981,16 +997,60 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>SMCI</t>
+          <t>SHC</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>SHOP</t>
+          <t>INCY</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>SMCI</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>APA</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>TRMB</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>TEAM</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>IOVA</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr"/>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>